<commit_message>
Phase 3: qa_pipeline, updated rag_config with dotenv, eval with chunk_top_k sweep
</commit_message>
<xml_diff>
--- a/tests/golden_set.xlsx
+++ b/tests/golden_set.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\sleman-one\projects\moc-agent\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6F7B96E-5B1D-4246-91D2-70162DE5C4EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB3C854A-62E9-4307-8D6A-9F9084AE2C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="150" yWindow="2895" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="495" yWindow="3240" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Golden Set" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="98">
   <si>
     <t>id</t>
   </si>
@@ -287,9 +287,6 @@
     <t>Can a merchant send me advertisements to my email without my permission?</t>
   </si>
   <si>
-    <t>نظام التجارة الإلكترونية + مشروع نظام حماية المستهلك</t>
-  </si>
-  <si>
     <t>لا. يشترط لإرسال إعلانات الحصول على موافقة المستهلك المسبقة والصريحة. ويُعد الإرسال دون إذن ممارسة تجارية مجحفة.</t>
   </si>
   <si>
@@ -317,7 +314,7 @@
     <t>المادة الثانية والأربعون</t>
   </si>
   <si>
-    <t>المادة العشرون (نظام التجارة الإلكترونية)</t>
+    <t>المادة العشرون: الإعلان الإلكتروني</t>
   </si>
 </sst>
 </file>
@@ -1089,7 +1086,7 @@
         <v>9</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>62</v>
@@ -1224,13 +1221,13 @@
         <v>87</v>
       </c>
       <c r="D21" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>51</v>
@@ -1252,10 +1249,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1263,7 +1260,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1271,7 +1268,7 @@
         <v>31</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1279,7 +1276,7 @@
         <v>51</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1287,7 +1284,7 @@
         <v>63</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1295,7 +1292,7 @@
         <v>85</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>